<commit_message>
Quiz tab redesign, practice content passes, lesson visuals engine
- Quiz tab: Ways to Play carousel, Quiz by Format grid (7 types + Hard Mode),
  Quiz by World cards, consistent surfaces, ripples, locked-card dialog,
  daily/quick sessions picked up front. Includes a TEMP quiz-reset icon in
  the toolbar (testing only).
- Practice and task-list cards use the shared ripple.
- Practice content passes for Worlds 9-16, lesson visual engine and standard.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CodeDo_Detailed_Explanation_Highlighted.xlsx
+++ b/CodeDo_Detailed_Explanation_Highlighted.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/apple/Desktop/PersonalProjects/CodeDoRN/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_1892E7E4111E9598D13DEA9C6D43793E7827F5A6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5ECBD8E-404B-9A44-83F3-B350B45996BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2775,10 +2775,10 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="45" customWidth="1"/>
-    <col min="3" max="3" width="20" customWidth="1"/>
-    <col min="4" max="4" width="70" customWidth="1"/>
-    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="2" max="2" width="33.1640625" customWidth="1"/>
+    <col min="3" max="3" width="1" customWidth="1"/>
+    <col min="4" max="5" width="1.33203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" hidden="1" customWidth="1"/>
     <col min="7" max="7" width="62" customWidth="1"/>
     <col min="8" max="8" width="24" customWidth="1"/>
     <col min="9" max="9" width="65" customWidth="1"/>

</xml_diff>